<commit_message>
fix: Medical mode skips dental pricing; update Factors.xlsx with extended 9x code rules
- In Medical mode, skip dental_pricing.json lookup and use medical_pricing.json
  directly. Previously, codes like 73221 that appear in both dental and medical
  pricing JSON were always matched as dental (isMedicalPricingMatch stayed false,
  factor not applied, dental prices used). Now Medical mode goes straight to
  medical pricing.
- Replace resources/Factors.xlsx with the new uploaded version which extends the
  Medical Services 'Starts With' rule from '1,2,3,4,5,6' to also cover 9x codes
  (91,92,93,94,95,96,98,99), enabling factor 1.3 for D001 on E&M and other 9x
  procedure codes at Truelife/Khabisi facilities.
</commit_message>
<xml_diff>
--- a/resources/Factors.xlsx
+++ b/resources/Factors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ray.james.TVI\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55624C1E-8E93-4126-ABB1-D987D6AFD1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{698ACF0B-385D-4C59-970D-90D79205C1F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1470" yWindow="1470" windowWidth="25290" windowHeight="13830" xr2:uid="{84C42952-5FA7-4B7D-9BCC-33BCBAD26808}"/>
   </bookViews>
@@ -140,9 +140,6 @@
     <t>99202, 99203, 99212, 99213</t>
   </si>
   <si>
-    <t>1, 2, 3, 4, 5, or 6</t>
-  </si>
-  <si>
     <t>Code Match Value</t>
   </si>
   <si>
@@ -168,6 +165,9 @@
   </si>
   <si>
     <t>Mednet (C004)</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 4, 5, 6, 91, 92, 93, 94,95, 96, 98, 99</t>
   </si>
 </sst>
 </file>
@@ -751,7 +751,7 @@
     <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.28515625" customWidth="1"/>
+    <col min="5" max="5" width="36.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
@@ -774,31 +774,31 @@
         <v>24</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>40</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>41</v>
-      </c>
-      <c r="L1" t="s">
-        <v>42</v>
       </c>
       <c r="P1" t="s">
         <v>19</v>
@@ -930,7 +930,7 @@
         <v>28</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F4" s="2">
         <v>1.3</v>
@@ -1185,7 +1185,7 @@
         <v>28</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F9" s="2">
         <v>1.3</v>
@@ -1434,7 +1434,7 @@
         <v>28</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F14" s="2">
         <v>1</v>

</xml_diff>